<commit_message>
Enhance OJT Masterlist Import/Export Functionality
- Added duplicate student number check during masterlist import to prevent overwriting existing records.
- Implemented a new function to delete masterlist entries based on school year and semester.
- Updated the export functionality to include additional filtering options for external masterlist exports.
- Improved user feedback on import operations, including summary of skipped duplicates and deletion results.
- Adjusted SQL queries to ensure proper handling of student numbers and masterlist data integrity.
</commit_message>
<xml_diff>
--- a/BioTern/assets/OJT MONITORING SY 25-26 External Students Template.xlsx
+++ b/BioTern/assets/OJT MONITORING SY 25-26 External Students Template.xlsx
@@ -1,13 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="External Students" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>BioTern</Application>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>BioTern</dc:creator>
+  <cp:lastModifiedBy>BioTern</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-05-01T23:08:13Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-05-01T23:08:13Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="2">
     <font>
@@ -50,7 +57,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="External Students" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:L199"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
@@ -134,7 +149,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t/>
+          <t>05-8531</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -196,7 +211,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t/>
+          <t>05-8377</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -259,7 +274,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t/>
+          <t>05-12346</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -321,7 +336,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t/>
+          <t>05-8969</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -383,7 +398,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t/>
+          <t>05-7262</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -756,7 +771,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t/>
+          <t>05-12346</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -880,7 +895,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t/>
+          <t>05-8969</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4177,7 +4192,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LEAñO, JOHN LEVY C.</t>
+          <t>LEAÃ±O, JOHN LEVY C.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -6311,7 +6326,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>MR. AARON BAÑARES</t>
+          <t>MR. AARON BAÃ‘ARES</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -7117,7 +7132,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>MR. AARON BAÑARES</t>
+          <t>MR. AARON BAÃ‘ARES</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7985,7 +8000,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>MR. AARON BAÑARES</t>
+          <t>MR. AARON BAÃ‘ARES</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8109,7 +8124,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>MR. AARON BAÑARES</t>
+          <t>MR. AARON BAÃ‘ARES</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8419,7 +8434,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>HON. FERCIVAL D. DELA PEÑA</t>
+          <t>HON. FERCIVAL D. DELA PEÃ‘A</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8915,7 +8930,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>HON. FERCIVAL D. DELA PEÑA</t>
+          <t>HON. FERCIVAL D. DELA PEÃ‘A</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8977,7 +8992,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>HON. FERCIVAL D. DELA PEÑA</t>
+          <t>HON. FERCIVAL D. DELA PEÃ‘A</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9101,7 +9116,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>HON. FERCIVAL D. DELA PEÑA</t>
+          <t>HON. FERCIVAL D. DELA PEÃ‘A</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -10031,7 +10046,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>HON. FERCIVAL D. DELA PEÑA</t>
+          <t>HON. FERCIVAL D. DELA PEÃ‘A</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10192,7 +10207,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>NUñEZ, JOHN PAULO D.</t>
+          <t>NUÃ±EZ, JOHN PAULO D.</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -10651,7 +10666,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>HON. FERCIVAL D. DELA PEÑA</t>
+          <t>HON. FERCIVAL D. DELA PEÃ‘A</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -10837,7 +10852,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>HON. FERCIVAL D. DELA PEÑA</t>
+          <t>HON. FERCIVAL D. DELA PEÃ‘A</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">

</xml_diff>